<commit_message>
Sync maestro and Apps Script catalogs with On/Off technology.
Co-authored-by: anibaloperacionesWes <anibaloperacionesWes@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mantenimiento_wes/MAESTRO_FORMULARIO_WES.xlsx
+++ b/mantenimiento_wes/MAESTRO_FORMULARIO_WES.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Puntos" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contactos" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tecnicos" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallas" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opciones" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Puntos" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Contactos" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Tecnicos" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Fallas" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Opciones" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -551,7 +551,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Generado: 2026-08-18 03:16</t>
+          <t>Generado: 2026-08-20 15:57</t>
         </is>
       </c>
     </row>
@@ -7976,7 +7976,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C65"/>
+  <dimension ref="A1:C66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -8229,12 +8229,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>estados_checklist</t>
+          <t>tecnologias</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>On/Off</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -8249,7 +8249,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Observación</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -8264,7 +8264,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Falla</t>
+          <t>Observación</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -8279,7 +8279,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Falla</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -8289,12 +8289,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>cir</t>
+          <t>estados_checklist</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Canalización 24V AC</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -8309,7 +8309,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Canalización 220V AC</t>
+          <t>Canalización 24V AC</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -8324,7 +8324,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Poste solar</t>
+          <t>Canalización 220V AC</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -8339,7 +8339,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Panel solar</t>
+          <t>Poste solar</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -8354,7 +8354,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Batería solar</t>
+          <t>Panel solar</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -8369,7 +8369,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Cargador solar</t>
+          <t>Batería solar</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -8384,7 +8384,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Router / Amplimax</t>
+          <t>Cargador solar</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -8399,7 +8399,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Conectividad App</t>
+          <t>Router / Amplimax</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -8414,7 +8414,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Fuente switching 12V</t>
+          <t>Conectividad App</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -8429,7 +8429,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Batería respaldo CIR</t>
+          <t>Fuente switching 12V</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -8444,7 +8444,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Estado exterior caja CIR</t>
+          <t>Batería respaldo CIR</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -8459,7 +8459,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Estado interior caja CIR</t>
+          <t>Estado exterior caja CIR</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -8474,7 +8474,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Enlace CIR</t>
+          <t>Estado interior caja CIR</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -8489,7 +8489,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Voltaje 12V DC CIR</t>
+          <t>Enlace CIR</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -8504,7 +8504,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Voltaje 9V DC CIR</t>
+          <t>Voltaje 12V DC CIR</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -8519,7 +8519,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Voltaje 5V DC CIR</t>
+          <t>Voltaje 9V DC CIR</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -8534,7 +8534,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Equipo ultrasónico</t>
+          <t>Voltaje 5V DC CIR</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -8549,7 +8549,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Transductores</t>
+          <t>Equipo ultrasónico</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -8564,7 +8564,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Sensor de pulso</t>
+          <t>Transductores</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -8574,12 +8574,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>cpa</t>
+          <t>cir</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Presurización cañerías</t>
+          <t>Sensor de pulso</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -8594,7 +8594,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Cámara albañilería</t>
+          <t>Presurización cañerías</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -8609,7 +8609,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Tapa metálica</t>
+          <t>Cámara albañilería</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Llaves de paso</t>
+          <t>Tapa metálica</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -8639,7 +8639,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Válvula presión alta</t>
+          <t>Llaves de paso</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -8654,7 +8654,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Válvula presión baja</t>
+          <t>Válvula presión alta</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -8669,7 +8669,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Válvula presión nocturna</t>
+          <t>Válvula presión baja</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -8684,7 +8684,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Solenoide válvula alta</t>
+          <t>Válvula presión nocturna</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -8699,7 +8699,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Solenoide válvula baja</t>
+          <t>Solenoide válvula alta</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -8714,7 +8714,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Solenoide válvula nocturna</t>
+          <t>Solenoide válvula baja</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -8729,7 +8729,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Func. presión alta</t>
+          <t>Solenoide válvula nocturna</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -8744,7 +8744,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Func. presión baja</t>
+          <t>Func. presión alta</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -8759,7 +8759,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Func. presión nocturna</t>
+          <t>Func. presión baja</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -8774,7 +8774,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Func. medidor</t>
+          <t>Func. presión nocturna</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -8784,12 +8784,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>sab</t>
+          <t>cpa</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Canalización 24V AC</t>
+          <t>Func. medidor</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -8804,7 +8804,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Canalización 220V AC</t>
+          <t>Canalización 24V AC</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Voltaje 12V DC</t>
+          <t>Canalización 220V AC</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -8834,7 +8834,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Voltaje 9V DC</t>
+          <t>Voltaje 12V DC</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -8849,7 +8849,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Voltaje 5V DC</t>
+          <t>Voltaje 9V DC</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -8864,7 +8864,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Temporización</t>
+          <t>Voltaje 5V DC</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -8879,7 +8879,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Sensores</t>
+          <t>Temporización</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -8894,7 +8894,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Presurización cañerías</t>
+          <t>Sensores</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -8909,7 +8909,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Llaves de paso</t>
+          <t>Presurización cañerías</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -8924,7 +8924,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Válvula solenoide</t>
+          <t>Llaves de paso</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -8939,7 +8939,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Tiempo de descarga</t>
+          <t>Válvula solenoide</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -8954,11 +8954,26 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Caudal urinario</t>
+          <t>Tiempo de descarga</t>
         </is>
       </c>
       <c r="C65" t="n">
         <v>64</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>sab</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Caudal urinario</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix contact autosave wiping CORMUP/RENCA generals and remove EYES.
Stop overwriting client-level Contactos rows from visits, dedupe punto
rows, restore David Campos and Renca corporación, and drop EYES tech.

Co-authored-by: anibaloperacionesWes <anibaloperacionesWes@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mantenimiento_wes/MAESTRO_FORMULARIO_WES.xlsx
+++ b/mantenimiento_wes/MAESTRO_FORMULARIO_WES.xlsx
@@ -551,7 +551,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Generado: 2026-08-20 15:57</t>
+          <t>Generado: 2026-08-20 17:29</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B156"/>
+  <dimension ref="A1:B121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -636,7 +636,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>INTERMODAL</t>
+          <t>MODULO ABC</t>
         </is>
       </c>
     </row>
@@ -648,7 +648,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>MODULO ABC</t>
+          <t>MODULO D</t>
         </is>
       </c>
     </row>
@@ -660,7 +660,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>MODULO D</t>
+          <t>MODULO E</t>
         </is>
       </c>
     </row>
@@ -672,7 +672,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>MODULO E</t>
+          <t>INTERMODAL</t>
         </is>
       </c>
     </row>
@@ -1351,24 +1351,24 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>ESTADIO ISRAELITA</t>
+          <t>FUNDO ZAPALLAR</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>MATRIS CHESTERTON</t>
+          <t>ESTANQUE INFERIOR</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>ESTADIO ISRAELITA</t>
+          <t>FUNDO ZAPALLAR</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>MATRIZ AV LAS CONDES</t>
+          <t>ETAPA 1</t>
         </is>
       </c>
     </row>
@@ -1380,7 +1380,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>ESTANQUE INFERIOR</t>
+          <t>ETAPA 1,2,3 Y 4</t>
         </is>
       </c>
     </row>
@@ -1392,7 +1392,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>ETAPA 1</t>
+          <t>ETAPA 1-4</t>
         </is>
       </c>
     </row>
@@ -1404,7 +1404,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>ETAPA 1,2,3 Y 4</t>
+          <t>ETAPA 2</t>
         </is>
       </c>
     </row>
@@ -1416,7 +1416,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>ETAPA 1-4</t>
+          <t>ETAPA 3</t>
         </is>
       </c>
     </row>
@@ -1428,7 +1428,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>ETAPA 2</t>
+          <t>ETAPA 5</t>
         </is>
       </c>
     </row>
@@ -1440,7 +1440,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>ETAPA 3</t>
+          <t>MATRIZ ESVAL</t>
         </is>
       </c>
     </row>
@@ -1452,1001 +1452,581 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>ETAPA 5</t>
+          <t>RIEGO LLENADO DE ESTANQUE ESVAL</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>FUNDO ZAPALLAR</t>
+          <t>LA FLORIDA</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>MATRIZ ESVAL</t>
+          <t>LICEO ALTO CORDILLERA</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>FUNDO ZAPALLAR</t>
+          <t>LA REINA</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>RIEGO LLENADO DE ESTANQUE ESVAL</t>
+          <t>EUGENIO MARIA DE HOSTOS</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>LAS CONDES</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>CDP PUENTE ALTO</t>
+          <t>FLEMING</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>LO VALLEDOR</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>COLINA 1</t>
+          <t>BARRIO NORTE</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>LO VALLEDOR</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>COLINA 2 RED SUR</t>
+          <t>POZO 1</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>LO VALLEDOR</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>COLINA 2 REDIMPULSION</t>
+          <t>PUERTA 1</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>MAE</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>CPA MODULO</t>
+          <t>BAÑO GUARDIAS</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>MAE</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>CPA OVALO</t>
+          <t>ESTANQUE  CARGA ESTANQUE SUR</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>MAE</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>CPF SAN MIGUEL MATRIZ PRINCIPAL</t>
+          <t>ESTANQUE NORTE LOCALES</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>MAE</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>CPF SAN MIGUEL SALA IMPULSION</t>
+          <t>PIZZA HUT</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>MAE</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>ESC. EL BOSQUE ADMINISTRACION</t>
+          <t>SALA DE BOMBAS ESTANQUE SUR</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>MAM</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>ESC. EL BOSQUE GENCHI ACADEMIA</t>
+          <t>MATRIZ BOULEVARD PASILLO TECNICO</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>MAM</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>ESC. OF ARTEMIO</t>
+          <t>MATRIZ SALIDA DE EMERGENCIA PASILLO N°1 ARROW</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>MAM</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>ESC. OF CARMEN</t>
+          <t>PLACA BANCARIA</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>MAM</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>ESCUELA ANDES DEL SUR</t>
+          <t>SALA DE BOMBAS FALABELLA</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>MAM</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>ESFORPEN BOSQUE ADMINISTRACION</t>
+          <t>SALA DE BOMBAS RIPLEY</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>MAQ</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>ESFORPEN BOSQUE GENCHI SIMULACION</t>
+          <t>ALIMENTACION DE BAÑOS</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>MAQ</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>MONITOREO MATRIZ PRINCIPAL MODULO</t>
+          <t>MATRIZ PRINCIPAL</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>GENCHI</t>
+          <t>MAQ</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>MONITOREO MATRIZ PRINCIPAL OVALO</t>
+          <t>RED DE INCENDIO</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>HEGC</t>
+          <t>NIDO</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>AGUA BLANDA</t>
+          <t>CONTROL NIDO</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>HEGC</t>
+          <t>NIDO</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>INTERCAMBIADOR 1</t>
+          <t>ELEMENTARY</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>HEGC</t>
+          <t>NIDO</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>INTERCAMBIADOR 2</t>
+          <t>ESTANQUE B</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>HEGC</t>
+          <t>NIDO</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>MATRIZ PRINCIPAL</t>
+          <t>ESTANQUE C</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>HEGC</t>
+          <t>NIDO</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>RETORNO OSMOSIS</t>
+          <t>HIGH SCHOOL</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>HEGC</t>
+          <t>NIDO</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>SALIDA OSMOSIS</t>
+          <t>PISCINA</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>LA FLORIDA</t>
+          <t>NIDO</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>LICEO ALTO CORDILLERA</t>
+          <t>POZO PROFUNDO</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>LA REINA</t>
+          <t>NIDO</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>EUGENIO MARIA DE HOSTOS</t>
+          <t>TEATRO</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>LAS CONDES</t>
+          <t>PAK</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>FLEMING</t>
+          <t>ANDEN 3-4 LOCALES GASTRONOMICOS</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>LO VALLEDOR</t>
+          <t>PAK</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>BARRIO NORTE</t>
+          <t>ANDEN 3-4 MATRIZ PRINCIPAL</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>LO VALLEDOR</t>
+          <t>PAK</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>POZO 1</t>
+          <t>ANDEN 3-4 RESTAURANTE</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>LO VALLEDOR</t>
+          <t>PAK</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>PUERTA 1</t>
+          <t>BAZAR GOURMET</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>MADECCO</t>
+          <t>PAK</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>CASINO</t>
+          <t>DISTRITO DE LUJO</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>MADECCO</t>
+          <t>PAK</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>ESTANQUE CISTERNA</t>
+          <t>DL KENNEDY</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>MADECCO</t>
+          <t>PAK</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>SAN NICOLAS</t>
+          <t>LLENADO DE PILETA</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>MADECCO</t>
+          <t>PAK</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>URETA COX</t>
+          <t>PILETA CASCADA</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>MAE</t>
+          <t>PAK</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>BAÑO GUARDIAS</t>
+          <t>SANDIA ANTIGUA</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>MAE</t>
+          <t>PAK</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>ESTANQUE  CARGA ESTANQUE SUR</t>
+          <t>SANDIA NUEVA</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>MAE</t>
+          <t>PROVIDENCIA</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>ESTANQUE NORTE LOCALES</t>
+          <t>CARMELA CARVAJAL</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>MAE</t>
+          <t>PROVIDENCIA</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>PIZZA HUT</t>
+          <t>LASTARRIA</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>MAE</t>
+          <t>PROVIDENCIA</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>SALA DE BOMBAS ESTANQUE SUR</t>
+          <t>LICEO JUAN PABLO DUARTE</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>MAM</t>
+          <t>PROVIDENCIA</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>MATRIZ BOULEVARD PASILLO TECNICO</t>
+          <t>LICEO N°7</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>MAM</t>
+          <t>RENCA</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>MATRIZ SALIDA DE EMERGENCIA PASILLO N°1 ARROW</t>
+          <t>ICCO</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>MAM</t>
+          <t>RENCA</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>PLACA BANCARIA</t>
+          <t>ICCP</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>MAM</t>
+          <t>RENCA</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>SALA DE BOMBAS FALABELLA</t>
+          <t>ESCUELA LO VELEZQUEZ</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>MAM</t>
+          <t>RENCA</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>SALA DE BOMBAS RIPLEY</t>
+          <t>GIMNASIO MUNICIPAL</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>MAQ</t>
+          <t>RENCA</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>ALIMENTACION DE BAÑOS</t>
+          <t>PISCINA MUNICIPAL</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>MAQ</t>
+          <t>UDD</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>MATRIZ PRINCIPAL</t>
+          <t>SALA DE BOMBAS EDIFICIO ¨O¨</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>MAQ</t>
+          <t>UDD</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
-        <is>
-          <t>RED DE INCENDIO</t>
-        </is>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" t="inlineStr">
-        <is>
-          <t>MOLYMET</t>
-        </is>
-      </c>
-      <c r="B122" t="inlineStr">
-        <is>
-          <t>CASA DE CAMBIO</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" t="inlineStr">
-        <is>
-          <t>MOLYMET</t>
-        </is>
-      </c>
-      <c r="B123" t="inlineStr">
-        <is>
-          <t>RIEGO</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" t="inlineStr">
-        <is>
-          <t>NIDO</t>
-        </is>
-      </c>
-      <c r="B124" t="inlineStr">
-        <is>
-          <t>CONTROL NIDO</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" t="inlineStr">
-        <is>
-          <t>NIDO</t>
-        </is>
-      </c>
-      <c r="B125" t="inlineStr">
-        <is>
-          <t>ELEMENTARY</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" t="inlineStr">
-        <is>
-          <t>NIDO</t>
-        </is>
-      </c>
-      <c r="B126" t="inlineStr">
-        <is>
-          <t>ESTANQUE B</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" t="inlineStr">
-        <is>
-          <t>NIDO</t>
-        </is>
-      </c>
-      <c r="B127" t="inlineStr">
-        <is>
-          <t>ESTANQUE C</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" t="inlineStr">
-        <is>
-          <t>NIDO</t>
-        </is>
-      </c>
-      <c r="B128" t="inlineStr">
-        <is>
-          <t>HIGH SCHOOL</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" t="inlineStr">
-        <is>
-          <t>NIDO</t>
-        </is>
-      </c>
-      <c r="B129" t="inlineStr">
-        <is>
-          <t>PISCINA</t>
-        </is>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" t="inlineStr">
-        <is>
-          <t>NIDO</t>
-        </is>
-      </c>
-      <c r="B130" t="inlineStr">
-        <is>
-          <t>POZO PROFUNDO</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" t="inlineStr">
-        <is>
-          <t>NIDO</t>
-        </is>
-      </c>
-      <c r="B131" t="inlineStr">
-        <is>
-          <t>TEATRO</t>
-        </is>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" t="inlineStr">
-        <is>
-          <t>PAE</t>
-        </is>
-      </c>
-      <c r="B132" t="inlineStr">
-        <is>
-          <t>ESTANQUE  CARGA ESTANQUE SUR</t>
-        </is>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" t="inlineStr">
-        <is>
-          <t>PAE</t>
-        </is>
-      </c>
-      <c r="B133" t="inlineStr">
-        <is>
-          <t>ESTANQUE NORTE LOCALES</t>
-        </is>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" t="inlineStr">
-        <is>
-          <t>PAE</t>
-        </is>
-      </c>
-      <c r="B134" t="inlineStr">
-        <is>
-          <t>KFC</t>
-        </is>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" t="inlineStr">
-        <is>
-          <t>PAE</t>
-        </is>
-      </c>
-      <c r="B135" t="inlineStr">
-        <is>
-          <t>PIZZA HUT</t>
-        </is>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" t="inlineStr">
-        <is>
-          <t>PAK</t>
-        </is>
-      </c>
-      <c r="B136" t="inlineStr">
-        <is>
-          <t>ANDEN 3-4 LOCALES GASTRONOMICOS</t>
-        </is>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" t="inlineStr">
-        <is>
-          <t>PAK</t>
-        </is>
-      </c>
-      <c r="B137" t="inlineStr">
-        <is>
-          <t>ANDEN 3-4 MATRIZ PRINCIPAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" t="inlineStr">
-        <is>
-          <t>PAK</t>
-        </is>
-      </c>
-      <c r="B138" t="inlineStr">
-        <is>
-          <t>ANDEN 3-4 RESTAURANTE</t>
-        </is>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" t="inlineStr">
-        <is>
-          <t>PAK</t>
-        </is>
-      </c>
-      <c r="B139" t="inlineStr">
-        <is>
-          <t>BAZAR GOURMET</t>
-        </is>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" t="inlineStr">
-        <is>
-          <t>PAK</t>
-        </is>
-      </c>
-      <c r="B140" t="inlineStr">
-        <is>
-          <t>DISTRITO DE LUJO</t>
-        </is>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" t="inlineStr">
-        <is>
-          <t>PAK</t>
-        </is>
-      </c>
-      <c r="B141" t="inlineStr">
-        <is>
-          <t>DL KENNEDY</t>
-        </is>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" t="inlineStr">
-        <is>
-          <t>PAK</t>
-        </is>
-      </c>
-      <c r="B142" t="inlineStr">
-        <is>
-          <t>LLENADO DE PILETA</t>
-        </is>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" t="inlineStr">
-        <is>
-          <t>PAK</t>
-        </is>
-      </c>
-      <c r="B143" t="inlineStr">
-        <is>
-          <t>PILETA CASCADA</t>
-        </is>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" t="inlineStr">
-        <is>
-          <t>PAK</t>
-        </is>
-      </c>
-      <c r="B144" t="inlineStr">
-        <is>
-          <t>SANDIA ANTIGUA</t>
-        </is>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" t="inlineStr">
-        <is>
-          <t>PAK</t>
-        </is>
-      </c>
-      <c r="B145" t="inlineStr">
-        <is>
-          <t>SANDIA NUEVA</t>
-        </is>
-      </c>
-    </row>
-    <row r="146">
-      <c r="A146" t="inlineStr">
-        <is>
-          <t>PROVIDENCIA</t>
-        </is>
-      </c>
-      <c r="B146" t="inlineStr">
-        <is>
-          <t>CARMELA CARVAJAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" t="inlineStr">
-        <is>
-          <t>PROVIDENCIA</t>
-        </is>
-      </c>
-      <c r="B147" t="inlineStr">
-        <is>
-          <t>LASTARRIA</t>
-        </is>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" t="inlineStr">
-        <is>
-          <t>PROVIDENCIA</t>
-        </is>
-      </c>
-      <c r="B148" t="inlineStr">
-        <is>
-          <t>LICEO JUAN PABLO DUARTE</t>
-        </is>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" t="inlineStr">
-        <is>
-          <t>PROVIDENCIA</t>
-        </is>
-      </c>
-      <c r="B149" t="inlineStr">
-        <is>
-          <t>LICEO N°7</t>
-        </is>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" t="inlineStr">
-        <is>
-          <t>RENCA</t>
-        </is>
-      </c>
-      <c r="B150" t="inlineStr">
-        <is>
-          <t>ESCUELA LO VELEZQUEZ</t>
-        </is>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" t="inlineStr">
-        <is>
-          <t>RENCA</t>
-        </is>
-      </c>
-      <c r="B151" t="inlineStr">
-        <is>
-          <t>GIMNASIO MUNICIPAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" t="inlineStr">
-        <is>
-          <t>RENCA</t>
-        </is>
-      </c>
-      <c r="B152" t="inlineStr">
-        <is>
-          <t>ICCO</t>
-        </is>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" t="inlineStr">
-        <is>
-          <t>RENCA</t>
-        </is>
-      </c>
-      <c r="B153" t="inlineStr">
-        <is>
-          <t>ICCP</t>
-        </is>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" t="inlineStr">
-        <is>
-          <t>RENCA</t>
-        </is>
-      </c>
-      <c r="B154" t="inlineStr">
-        <is>
-          <t>PISCINA MUNICIPAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" t="inlineStr">
-        <is>
-          <t>UDD</t>
-        </is>
-      </c>
-      <c r="B155" t="inlineStr">
-        <is>
-          <t>SALA DE BOMBAS EDIFICIO ¨O¨</t>
-        </is>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" t="inlineStr">
-        <is>
-          <t>UDD</t>
-        </is>
-      </c>
-      <c r="B156" t="inlineStr">
         <is>
           <t>SALA DE BOMBAS HONDURAS</t>
         </is>
@@ -2463,7 +2043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G146"/>
+  <dimension ref="A1:G151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4377,19 +3957,11 @@
           <t>general</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>Fernanda Rojas</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>Líder de Innovación en Sustentabilidad</t>
-        </is>
-      </c>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr">
         <is>
-          <t>fernanda.rojas@renca.cl</t>
+          <t>Fabiola.Fuentes@sleplosparques.gob.cl</t>
         </is>
       </c>
       <c r="G63" t="inlineStr"/>
@@ -7036,6 +6608,171 @@
         </is>
       </c>
       <c r="G146" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>RENCA</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>ESCUELA LO VELEZQUEZ</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>punto</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Fabiola Fuentes</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>Jefa de infraestructura</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>andrea.romero@sleplosparques.gob.cl</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>RENCA</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>ICCO</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>punto</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Fabiola Fuentes</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>Jefa de infraestructura</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>maximiliano.gabarroche@sleplosparques.gob.cl</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>RENCA</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>ICCP</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>punto</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Fabiola Fuentes</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Jefa de infraestructura</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>Patricio.Diaz@sleplosparques.gob.cl</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>RENCA</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>GIMNASIO MUNICIPAL</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>punto</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Juan Erazo</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>Encargado de mantenimiento</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>juan.erazo@renca.cl</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr"/>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>RENCA</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>PISCINA MUNICIPAL</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>punto</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Juan Erazo</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>Encargado de mantenimiento</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>juan.erazo@renca.cl</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7976,7 +7713,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C66"/>
+  <dimension ref="A1:C65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -8189,7 +7926,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>EYES</t>
+          <t>CPA</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -8204,7 +7941,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CPA</t>
+          <t>CIR</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -8219,7 +7956,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CIR</t>
+          <t>On/Off</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -8229,12 +7966,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>tecnologias</t>
+          <t>estados_checklist</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>On/Off</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -8249,7 +7986,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Observación</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -8264,7 +8001,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Observación</t>
+          <t>Falla</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -8279,7 +8016,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Falla</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -8289,12 +8026,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>estados_checklist</t>
+          <t>cir</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Canalización 24V AC</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -8309,7 +8046,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Canalización 24V AC</t>
+          <t>Canalización 220V AC</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -8324,7 +8061,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Canalización 220V AC</t>
+          <t>Poste solar</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -8339,7 +8076,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Poste solar</t>
+          <t>Panel solar</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -8354,7 +8091,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Panel solar</t>
+          <t>Batería solar</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -8369,7 +8106,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Batería solar</t>
+          <t>Cargador solar</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -8384,7 +8121,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Cargador solar</t>
+          <t>Router / Amplimax</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -8399,7 +8136,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Router / Amplimax</t>
+          <t>Conectividad App</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -8414,7 +8151,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Conectividad App</t>
+          <t>Fuente switching 12V</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -8429,7 +8166,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Fuente switching 12V</t>
+          <t>Batería respaldo CIR</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -8444,7 +8181,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Batería respaldo CIR</t>
+          <t>Estado exterior caja CIR</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -8459,7 +8196,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Estado exterior caja CIR</t>
+          <t>Estado interior caja CIR</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -8474,7 +8211,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Estado interior caja CIR</t>
+          <t>Enlace CIR</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -8489,7 +8226,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Enlace CIR</t>
+          <t>Voltaje 12V DC CIR</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -8504,7 +8241,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Voltaje 12V DC CIR</t>
+          <t>Voltaje 9V DC CIR</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -8519,7 +8256,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Voltaje 9V DC CIR</t>
+          <t>Voltaje 5V DC CIR</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -8534,7 +8271,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Voltaje 5V DC CIR</t>
+          <t>Equipo ultrasónico</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -8549,7 +8286,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Equipo ultrasónico</t>
+          <t>Transductores</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -8564,7 +8301,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Transductores</t>
+          <t>Sensor de pulso</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -8574,12 +8311,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>cir</t>
+          <t>cpa</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Sensor de pulso</t>
+          <t>Presurización cañerías</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -8594,7 +8331,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Presurización cañerías</t>
+          <t>Cámara albañilería</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -8609,7 +8346,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Cámara albañilería</t>
+          <t>Tapa metálica</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -8624,7 +8361,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Tapa metálica</t>
+          <t>Llaves de paso</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -8639,7 +8376,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Llaves de paso</t>
+          <t>Válvula presión alta</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -8654,7 +8391,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Válvula presión alta</t>
+          <t>Válvula presión baja</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -8669,7 +8406,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Válvula presión baja</t>
+          <t>Válvula presión nocturna</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -8684,7 +8421,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Válvula presión nocturna</t>
+          <t>Solenoide válvula alta</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -8699,7 +8436,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Solenoide válvula alta</t>
+          <t>Solenoide válvula baja</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -8714,7 +8451,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Solenoide válvula baja</t>
+          <t>Solenoide válvula nocturna</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -8729,7 +8466,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Solenoide válvula nocturna</t>
+          <t>Func. presión alta</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -8744,7 +8481,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Func. presión alta</t>
+          <t>Func. presión baja</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -8759,7 +8496,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Func. presión baja</t>
+          <t>Func. presión nocturna</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -8774,7 +8511,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Func. presión nocturna</t>
+          <t>Func. medidor</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -8784,12 +8521,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>cpa</t>
+          <t>sab</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Func. medidor</t>
+          <t>Canalización 24V AC</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -8804,7 +8541,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Canalización 24V AC</t>
+          <t>Canalización 220V AC</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -8819,7 +8556,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Canalización 220V AC</t>
+          <t>Voltaje 12V DC</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -8834,7 +8571,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Voltaje 12V DC</t>
+          <t>Voltaje 9V DC</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -8849,7 +8586,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Voltaje 9V DC</t>
+          <t>Voltaje 5V DC</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -8864,7 +8601,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Voltaje 5V DC</t>
+          <t>Temporización</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -8879,7 +8616,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Temporización</t>
+          <t>Sensores</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -8894,7 +8631,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Sensores</t>
+          <t>Presurización cañerías</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -8909,7 +8646,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Presurización cañerías</t>
+          <t>Llaves de paso</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -8924,7 +8661,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Llaves de paso</t>
+          <t>Válvula solenoide</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -8939,7 +8676,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Válvula solenoide</t>
+          <t>Tiempo de descarga</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -8954,26 +8691,11 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Tiempo de descarga</t>
+          <t>Caudal urinario</t>
         </is>
       </c>
       <c r="C65" t="n">
         <v>64</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>sab</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>Caudal urinario</t>
-        </is>
-      </c>
-      <c r="C66" t="n">
-        <v>65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>